<commit_message>
test(preview): match only real Worker use and add a module-path hostile link (ENG-3594)
</commit_message>
<xml_diff>
--- a/e2e/document-preview/fixtures/xlsx/hostile.xlsx
+++ b/e2e/document-preview/fixtures/xlsx/hostile.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Kind</t>
   </si>
@@ -33,6 +33,9 @@
   </si>
   <si>
     <t xml:space="preserve">harness origin link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">harness module link</t>
   </si>
   <si>
     <t xml:space="preserve">localhost link</t>
@@ -91,7 +94,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -159,11 +162,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
-      </c>
-      <c r="B9" t="str">
-        <f>HYPERLINK("https://example.com/xlsx-formula","formula link")</f>
-        <v>formula link</v>
       </c>
     </row>
     <row r="10">
@@ -171,8 +173,8 @@
         <v>11</v>
       </c>
       <c r="B10" t="str">
-        <f>WEBSERVICE("https://example.com/xlsx-webservice")</f>
-        <v>web service value</v>
+        <f>HYPERLINK("https://example.com/xlsx-formula","formula link")</f>
+        <v>formula link</v>
       </c>
     </row>
     <row r="11">
@@ -180,21 +182,22 @@
         <v>12</v>
       </c>
       <c r="B11" t="str">
-        <f>[1]Prices!A1</f>
-        <v>external value</v>
+        <f>WEBSERVICE("https://example.com/xlsx-webservice")</f>
+        <v>web service value</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" t="s">
-        <v>14</v>
+      <c r="B12" t="str">
+        <f>[1]Prices!A1</f>
+        <v>external value</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -202,10 +205,18 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -217,6 +228,7 @@
     <hyperlink ref="B6" r:id="rId5"/>
     <hyperlink ref="B7" r:id="rId6"/>
     <hyperlink ref="B8" r:id="rId7"/>
+    <hyperlink ref="B9" r:id="rId8"/>
   </hyperlinks>
 </worksheet>
 </file>
@@ -227,7 +239,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2">

</xml_diff>